<commit_message>
correcion de caja con el wasap
</commit_message>
<xml_diff>
--- a/public/formats/persons.xlsx
+++ b/public/formats/persons.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brayan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sdrimsac\public\formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B3707C-D513-4384-B0B4-721AF4AEEECF}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641DD7BB-523A-4C79-BB81-364ECAF2C3C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>Número de documento</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t>Juan Pinedo</t>
+  </si>
+  <si>
+    <t>seller</t>
   </si>
 </sst>
 </file>
@@ -395,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
@@ -409,7 +412,7 @@
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -437,8 +440,11 @@
       <c r="I1" t="s">
         <v>7</v>
       </c>
+      <c r="J1" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -450,7 +456,7 @@
       </c>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>6</v>
       </c>

</xml_diff>